<commit_message>
Apply min tilt only when gap=0 in peer mode
</commit_message>
<xml_diff>
--- a/TAA_Dashboard.xlsx
+++ b/TAA_Dashboard.xlsx
@@ -1010,7 +1010,7 @@
         <v/>
       </c>
       <c r="K22" s="16">
-        <f>MAX(ABS(G22)*I22, J22)</f>
+        <f>IF(G22=0, J22, ABS(G22)*I22)</f>
         <v/>
       </c>
       <c r="L22" s="17">
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="K23" s="16">
-        <f>MAX(ABS(G23)*I23, J23)</f>
+        <f>IF(G23=0, J23, ABS(G23)*I23)</f>
         <v/>
       </c>
       <c r="L23" s="17">
@@ -1126,7 +1126,7 @@
         <v/>
       </c>
       <c r="K24" s="16">
-        <f>MAX(ABS(G24)*I24, J24)</f>
+        <f>IF(G24=0, J24, ABS(G24)*I24)</f>
         <v/>
       </c>
       <c r="L24" s="17">
@@ -1184,7 +1184,7 @@
         <v/>
       </c>
       <c r="K25" s="16">
-        <f>MAX(ABS(G25)*I25, J25)</f>
+        <f>IF(G25=0, J25, ABS(G25)*I25)</f>
         <v/>
       </c>
       <c r="L25" s="17">
@@ -1242,7 +1242,7 @@
         <v/>
       </c>
       <c r="K26" s="16">
-        <f>MAX(ABS(G26)*I26, J26)</f>
+        <f>IF(G26=0, J26, ABS(G26)*I26)</f>
         <v/>
       </c>
       <c r="L26" s="17">
@@ -1300,7 +1300,7 @@
         <v/>
       </c>
       <c r="K27" s="16">
-        <f>MAX(ABS(G27)*I27, J27)</f>
+        <f>IF(G27=0, J27, ABS(G27)*I27)</f>
         <v/>
       </c>
       <c r="L27" s="17">
@@ -1358,7 +1358,7 @@
         <v/>
       </c>
       <c r="K28" s="16">
-        <f>MAX(ABS(G28)*I28, J28)</f>
+        <f>IF(G28=0, J28, ABS(G28)*I28)</f>
         <v/>
       </c>
       <c r="L28" s="17">
@@ -1416,7 +1416,7 @@
         <v/>
       </c>
       <c r="K29" s="16">
-        <f>MAX(ABS(G29)*I29, J29)</f>
+        <f>IF(G29=0, J29, ABS(G29)*I29)</f>
         <v/>
       </c>
       <c r="L29" s="17">
@@ -1744,7 +1744,7 @@
     <row r="49">
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>5. Tilt_i = MAX( |Gap_i| × Damping_i,  Peer_i × Min Tilt Rate )</t>
+          <t>5. Tilt_i = |Gap_i| × Damping_i  (gap=0이면 Peer_i × Min Tilt Rate)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Excel layout and use VLOOKUP for signal mapping
</commit_message>
<xml_diff>
--- a/TAA_Dashboard.xlsx
+++ b/TAA_Dashboard.xlsx
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,11 +136,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -547,23 +550,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O53"/>
+  <dimension ref="B1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -600,13 +603,15 @@
           <t>← 0~1 (보수적 → 적극적)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Strong OW</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>2</v>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>TAA</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -623,13 +628,13 @@
           <t>← 0~1 (0=강한억제, 1=억제없음)</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Overweight</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>1</v>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Strong OW</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -646,1131 +651,1141 @@
           <t>← gap=0일 때 최소 Tilt 보장율</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Overweight</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I7" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="H7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I8" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="H8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Strong UW</t>
         </is>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I9" s="8" t="n">
         <v>-2</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Region Inputs</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="7" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>SAA(%)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Peer(%)</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>TAA</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E12" s="11" t="n">
         <v>45.5</v>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>유럽</t>
         </is>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E13" s="11" t="n">
         <v>12.6</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>일본</t>
         </is>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E14" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <v>2.1</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E15" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D16" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E16" s="11" t="n">
         <v>2.1</v>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>기타</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <v>1.4</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E17" s="11" t="n">
         <v>2.8</v>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>채권</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E18" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>채권</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E19" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>SAA</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Peer</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Aligned?</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Damping</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Min Tilt</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Tilt</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>Adj</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
+      <c r="M22" s="6" t="inlineStr">
         <is>
           <t>Raw</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="N22" s="6" t="inlineStr">
         <is>
           <t>Final(%)</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>vs Peer</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="12">
-        <f>B11</f>
-        <v/>
-      </c>
-      <c r="C22" s="13">
-        <f>C11</f>
-        <v/>
-      </c>
-      <c r="D22" s="14">
-        <f>D11</f>
-        <v/>
-      </c>
-      <c r="E22" s="14">
-        <f>E11</f>
-        <v/>
-      </c>
-      <c r="F22" s="15">
-        <f>IF(F11="Strong OW",2,IF(F11="Overweight",1,IF(F11="Neutral",0,IF(F11="Underweight",-1,IF(F11="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>D22-E22</f>
-        <v/>
-      </c>
-      <c r="H22" s="15">
-        <f>IF(F22*G22&gt;=0,1,0)</f>
-        <v/>
-      </c>
-      <c r="I22" s="16">
-        <f>H22*(1-$C$5)+$C$5</f>
-        <v/>
-      </c>
-      <c r="J22" s="16">
-        <f>E22*$C$6</f>
-        <v/>
-      </c>
-      <c r="K22" s="16">
-        <f>IF(G22=0, J22, ABS(G22)*I22)</f>
-        <v/>
-      </c>
-      <c r="L22" s="17">
-        <f>$C$4*F22*K22</f>
-        <v/>
-      </c>
-      <c r="M22" s="16">
-        <f>MAX(E22+L22, 1.0)</f>
-        <v/>
-      </c>
-      <c r="N22" s="18">
-        <f>ROUND(M22/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O22" s="17">
-        <f>ROUND(N22-E22, 2)</f>
-        <v/>
-      </c>
-    </row>
     <row r="23">
-      <c r="B23" s="12">
+      <c r="B23" s="13">
         <f>B12</f>
         <v/>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="14">
         <f>C12</f>
         <v/>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="15">
         <f>D12</f>
         <v/>
       </c>
-      <c r="E23" s="14">
+      <c r="E23" s="15">
         <f>E12</f>
         <v/>
       </c>
-      <c r="F23" s="15">
-        <f>IF(F12="Strong OW",2,IF(F12="Overweight",1,IF(F12="Neutral",0,IF(F12="Underweight",-1,IF(F12="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
+      <c r="F23" s="16">
+        <f>VLOOKUP(F12,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G23" s="17">
         <f>D23-E23</f>
         <v/>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="16">
         <f>IF(F23*G23&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I23" s="16">
+      <c r="I23" s="17">
         <f>H23*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="17">
         <f>E23*$C$6</f>
         <v/>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="17">
         <f>IF(G23=0, J23, ABS(G23)*I23)</f>
         <v/>
       </c>
-      <c r="L23" s="17">
+      <c r="L23" s="18">
         <f>$C$4*F23*K23</f>
         <v/>
       </c>
-      <c r="M23" s="16">
+      <c r="M23" s="17">
         <f>MAX(E23+L23, 1.0)</f>
         <v/>
       </c>
-      <c r="N23" s="18">
-        <f>ROUND(M23/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O23" s="17">
+      <c r="N23" s="19">
+        <f>ROUND(M23/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O23" s="18">
         <f>ROUND(N23-E23, 2)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="12">
+      <c r="B24" s="13">
         <f>B13</f>
         <v/>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="14">
         <f>C13</f>
         <v/>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="15">
         <f>D13</f>
         <v/>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="15">
         <f>E13</f>
         <v/>
       </c>
-      <c r="F24" s="15">
-        <f>IF(F13="Strong OW",2,IF(F13="Overweight",1,IF(F13="Neutral",0,IF(F13="Underweight",-1,IF(F13="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
+      <c r="F24" s="16">
+        <f>VLOOKUP(F13,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G24" s="17">
         <f>D24-E24</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="16">
         <f>IF(F24*G24&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I24" s="16">
+      <c r="I24" s="17">
         <f>H24*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="17">
         <f>E24*$C$6</f>
         <v/>
       </c>
-      <c r="K24" s="16">
+      <c r="K24" s="17">
         <f>IF(G24=0, J24, ABS(G24)*I24)</f>
         <v/>
       </c>
-      <c r="L24" s="17">
+      <c r="L24" s="18">
         <f>$C$4*F24*K24</f>
         <v/>
       </c>
-      <c r="M24" s="16">
+      <c r="M24" s="17">
         <f>MAX(E24+L24, 1.0)</f>
         <v/>
       </c>
-      <c r="N24" s="18">
-        <f>ROUND(M24/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O24" s="17">
+      <c r="N24" s="19">
+        <f>ROUND(M24/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O24" s="18">
         <f>ROUND(N24-E24, 2)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="12">
+      <c r="B25" s="13">
         <f>B14</f>
         <v/>
       </c>
-      <c r="C25" s="13">
+      <c r="C25" s="14">
         <f>C14</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="15">
         <f>D14</f>
         <v/>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="15">
         <f>E14</f>
         <v/>
       </c>
-      <c r="F25" s="15">
-        <f>IF(F14="Strong OW",2,IF(F14="Overweight",1,IF(F14="Neutral",0,IF(F14="Underweight",-1,IF(F14="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
+      <c r="F25" s="16">
+        <f>VLOOKUP(F14,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G25" s="17">
         <f>D25-E25</f>
         <v/>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="16">
         <f>IF(F25*G25&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I25" s="16">
+      <c r="I25" s="17">
         <f>H25*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J25" s="16">
+      <c r="J25" s="17">
         <f>E25*$C$6</f>
         <v/>
       </c>
-      <c r="K25" s="16">
+      <c r="K25" s="17">
         <f>IF(G25=0, J25, ABS(G25)*I25)</f>
         <v/>
       </c>
-      <c r="L25" s="17">
+      <c r="L25" s="18">
         <f>$C$4*F25*K25</f>
         <v/>
       </c>
-      <c r="M25" s="16">
+      <c r="M25" s="17">
         <f>MAX(E25+L25, 1.0)</f>
         <v/>
       </c>
-      <c r="N25" s="18">
-        <f>ROUND(M25/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O25" s="17">
+      <c r="N25" s="19">
+        <f>ROUND(M25/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O25" s="18">
         <f>ROUND(N25-E25, 2)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="12">
+      <c r="B26" s="13">
         <f>B15</f>
         <v/>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="14">
         <f>C15</f>
         <v/>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="15">
         <f>D15</f>
         <v/>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="15">
         <f>E15</f>
         <v/>
       </c>
-      <c r="F26" s="15">
-        <f>IF(F15="Strong OW",2,IF(F15="Overweight",1,IF(F15="Neutral",0,IF(F15="Underweight",-1,IF(F15="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
+      <c r="F26" s="16">
+        <f>VLOOKUP(F15,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G26" s="17">
         <f>D26-E26</f>
         <v/>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="16">
         <f>IF(F26*G26&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I26" s="16">
+      <c r="I26" s="17">
         <f>H26*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="17">
         <f>E26*$C$6</f>
         <v/>
       </c>
-      <c r="K26" s="16">
+      <c r="K26" s="17">
         <f>IF(G26=0, J26, ABS(G26)*I26)</f>
         <v/>
       </c>
-      <c r="L26" s="17">
+      <c r="L26" s="18">
         <f>$C$4*F26*K26</f>
         <v/>
       </c>
-      <c r="M26" s="16">
+      <c r="M26" s="17">
         <f>MAX(E26+L26, 1.0)</f>
         <v/>
       </c>
-      <c r="N26" s="18">
-        <f>ROUND(M26/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O26" s="17">
+      <c r="N26" s="19">
+        <f>ROUND(M26/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O26" s="18">
         <f>ROUND(N26-E26, 2)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="12">
+      <c r="B27" s="13">
         <f>B16</f>
         <v/>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="14">
         <f>C16</f>
         <v/>
       </c>
-      <c r="D27" s="14">
+      <c r="D27" s="15">
         <f>D16</f>
         <v/>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="15">
         <f>E16</f>
         <v/>
       </c>
-      <c r="F27" s="15">
-        <f>IF(F16="Strong OW",2,IF(F16="Overweight",1,IF(F16="Neutral",0,IF(F16="Underweight",-1,IF(F16="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
+      <c r="F27" s="16">
+        <f>VLOOKUP(F16,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G27" s="17">
         <f>D27-E27</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="16">
         <f>IF(F27*G27&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I27" s="16">
+      <c r="I27" s="17">
         <f>H27*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J27" s="16">
+      <c r="J27" s="17">
         <f>E27*$C$6</f>
         <v/>
       </c>
-      <c r="K27" s="16">
+      <c r="K27" s="17">
         <f>IF(G27=0, J27, ABS(G27)*I27)</f>
         <v/>
       </c>
-      <c r="L27" s="17">
+      <c r="L27" s="18">
         <f>$C$4*F27*K27</f>
         <v/>
       </c>
-      <c r="M27" s="16">
+      <c r="M27" s="17">
         <f>MAX(E27+L27, 1.0)</f>
         <v/>
       </c>
-      <c r="N27" s="18">
-        <f>ROUND(M27/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O27" s="17">
+      <c r="N27" s="19">
+        <f>ROUND(M27/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O27" s="18">
         <f>ROUND(N27-E27, 2)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="12">
+      <c r="B28" s="13">
         <f>B17</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C17</f>
         <v/>
       </c>
-      <c r="D28" s="14">
+      <c r="D28" s="15">
         <f>D17</f>
         <v/>
       </c>
-      <c r="E28" s="14">
+      <c r="E28" s="15">
         <f>E17</f>
         <v/>
       </c>
-      <c r="F28" s="15">
-        <f>IF(F17="Strong OW",2,IF(F17="Overweight",1,IF(F17="Neutral",0,IF(F17="Underweight",-1,IF(F17="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
+      <c r="F28" s="16">
+        <f>VLOOKUP(F17,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G28" s="17">
         <f>D28-E28</f>
         <v/>
       </c>
-      <c r="H28" s="15">
+      <c r="H28" s="16">
         <f>IF(F28*G28&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I28" s="16">
+      <c r="I28" s="17">
         <f>H28*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J28" s="16">
+      <c r="J28" s="17">
         <f>E28*$C$6</f>
         <v/>
       </c>
-      <c r="K28" s="16">
+      <c r="K28" s="17">
         <f>IF(G28=0, J28, ABS(G28)*I28)</f>
         <v/>
       </c>
-      <c r="L28" s="17">
+      <c r="L28" s="18">
         <f>$C$4*F28*K28</f>
         <v/>
       </c>
-      <c r="M28" s="16">
+      <c r="M28" s="17">
         <f>MAX(E28+L28, 1.0)</f>
         <v/>
       </c>
-      <c r="N28" s="18">
-        <f>ROUND(M28/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O28" s="17">
+      <c r="N28" s="19">
+        <f>ROUND(M28/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O28" s="18">
         <f>ROUND(N28-E28, 2)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="12">
+      <c r="B29" s="13">
         <f>B18</f>
         <v/>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="14">
         <f>C18</f>
         <v/>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="15">
         <f>D18</f>
         <v/>
       </c>
-      <c r="E29" s="14">
+      <c r="E29" s="15">
         <f>E18</f>
         <v/>
       </c>
-      <c r="F29" s="15">
-        <f>IF(F18="Strong OW",2,IF(F18="Overweight",1,IF(F18="Neutral",0,IF(F18="Underweight",-1,IF(F18="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
+      <c r="F29" s="16">
+        <f>VLOOKUP(F18,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G29" s="17">
         <f>D29-E29</f>
         <v/>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="16">
         <f>IF(F29*G29&gt;=0,1,0)</f>
         <v/>
       </c>
-      <c r="I29" s="16">
+      <c r="I29" s="17">
         <f>H29*(1-$C$5)+$C$5</f>
         <v/>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="17">
         <f>E29*$C$6</f>
         <v/>
       </c>
-      <c r="K29" s="16">
+      <c r="K29" s="17">
         <f>IF(G29=0, J29, ABS(G29)*I29)</f>
         <v/>
       </c>
-      <c r="L29" s="17">
+      <c r="L29" s="18">
         <f>$C$4*F29*K29</f>
         <v/>
       </c>
-      <c r="M29" s="16">
+      <c r="M29" s="17">
         <f>MAX(E29+L29, 1.0)</f>
         <v/>
       </c>
-      <c r="N29" s="18">
-        <f>ROUND(M29/SUM(M22:M29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="O29" s="17">
+      <c r="N29" s="19">
+        <f>ROUND(M29/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O29" s="18">
         <f>ROUND(N29-E29, 2)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B30" s="13">
+        <f>B19</f>
+        <v/>
+      </c>
+      <c r="C30" s="14">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="F30" s="16">
+        <f>VLOOKUP(F19,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G30" s="17">
+        <f>D30-E30</f>
+        <v/>
+      </c>
+      <c r="H30" s="16">
+        <f>IF(F30*G30&gt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="I30" s="17">
+        <f>H30*(1-$C$5)+$C$5</f>
+        <v/>
+      </c>
+      <c r="J30" s="17">
+        <f>E30*$C$6</f>
+        <v/>
+      </c>
+      <c r="K30" s="17">
+        <f>IF(G30=0, J30, ABS(G30)*I30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="18">
+        <f>$C$4*F30*K30</f>
+        <v/>
+      </c>
+      <c r="M30" s="17">
+        <f>MAX(E30+L30, 1.0)</f>
+        <v/>
+      </c>
+      <c r="N30" s="19">
+        <f>ROUND(M30/SUM(M23:M30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="O30" s="18">
+        <f>ROUND(N30-E30, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D30" s="20">
-        <f>SUM(D22:D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="20">
-        <f>SUM(E22:E29)</f>
-        <v/>
-      </c>
-      <c r="M30" s="20">
-        <f>SUM(M22:M29)</f>
-        <v/>
-      </c>
-      <c r="N30" s="20">
-        <f>SUM(N22:N29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="2" t="inlineStr">
+      <c r="D31" s="21">
+        <f>SUM(D23:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="21">
+        <f>SUM(E23:E30)</f>
+        <v/>
+      </c>
+      <c r="M31" s="21">
+        <f>SUM(M23:M30)</f>
+        <v/>
+      </c>
+      <c r="N31" s="21">
+        <f>SUM(N23:N30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Range (허용 범위)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Final(%)</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Half Width</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Low(%)</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>High(%)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="12">
-        <f>B22</f>
-        <v/>
-      </c>
-      <c r="C34" s="13">
-        <f>C22</f>
-        <v/>
-      </c>
-      <c r="D34" s="21">
-        <f>N22</f>
-        <v/>
-      </c>
-      <c r="E34" s="14">
-        <f>IF(D34&gt;=20, 7.5, IF(D34&gt;=10, 5.0, 2.5))</f>
-        <v/>
-      </c>
-      <c r="F34" s="22">
-        <f>ROUND(MAX(D34-E34, 0), 2)</f>
-        <v/>
-      </c>
-      <c r="G34" s="22">
-        <f>ROUND(D34+E34, 2)</f>
-        <v/>
-      </c>
-    </row>
     <row r="35">
-      <c r="B35" s="12">
+      <c r="B35" s="13">
         <f>B23</f>
         <v/>
       </c>
-      <c r="C35" s="13">
+      <c r="C35" s="14">
         <f>C23</f>
         <v/>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="22">
         <f>N23</f>
         <v/>
       </c>
-      <c r="E35" s="14">
+      <c r="E35" s="15">
         <f>IF(D35&gt;=20, 7.5, IF(D35&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F35" s="22">
+      <c r="F35" s="23">
         <f>ROUND(MAX(D35-E35, 0), 2)</f>
         <v/>
       </c>
-      <c r="G35" s="22">
+      <c r="G35" s="23">
         <f>ROUND(D35+E35, 2)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="12">
+      <c r="B36" s="13">
         <f>B24</f>
         <v/>
       </c>
-      <c r="C36" s="13">
+      <c r="C36" s="14">
         <f>C24</f>
         <v/>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="22">
         <f>N24</f>
         <v/>
       </c>
-      <c r="E36" s="14">
+      <c r="E36" s="15">
         <f>IF(D36&gt;=20, 7.5, IF(D36&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F36" s="22">
+      <c r="F36" s="23">
         <f>ROUND(MAX(D36-E36, 0), 2)</f>
         <v/>
       </c>
-      <c r="G36" s="22">
+      <c r="G36" s="23">
         <f>ROUND(D36+E36, 2)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="12">
+      <c r="B37" s="13">
         <f>B25</f>
         <v/>
       </c>
-      <c r="C37" s="13">
+      <c r="C37" s="14">
         <f>C25</f>
         <v/>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="22">
         <f>N25</f>
         <v/>
       </c>
-      <c r="E37" s="14">
+      <c r="E37" s="15">
         <f>IF(D37&gt;=20, 7.5, IF(D37&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="23">
         <f>ROUND(MAX(D37-E37, 0), 2)</f>
         <v/>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="23">
         <f>ROUND(D37+E37, 2)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="12">
+      <c r="B38" s="13">
         <f>B26</f>
         <v/>
       </c>
-      <c r="C38" s="13">
+      <c r="C38" s="14">
         <f>C26</f>
         <v/>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="22">
         <f>N26</f>
         <v/>
       </c>
-      <c r="E38" s="14">
+      <c r="E38" s="15">
         <f>IF(D38&gt;=20, 7.5, IF(D38&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F38" s="22">
+      <c r="F38" s="23">
         <f>ROUND(MAX(D38-E38, 0), 2)</f>
         <v/>
       </c>
-      <c r="G38" s="22">
+      <c r="G38" s="23">
         <f>ROUND(D38+E38, 2)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="12">
+      <c r="B39" s="13">
         <f>B27</f>
         <v/>
       </c>
-      <c r="C39" s="13">
+      <c r="C39" s="14">
         <f>C27</f>
         <v/>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="22">
         <f>N27</f>
         <v/>
       </c>
-      <c r="E39" s="14">
+      <c r="E39" s="15">
         <f>IF(D39&gt;=20, 7.5, IF(D39&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="23">
         <f>ROUND(MAX(D39-E39, 0), 2)</f>
         <v/>
       </c>
-      <c r="G39" s="22">
+      <c r="G39" s="23">
         <f>ROUND(D39+E39, 2)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="12">
+      <c r="B40" s="13">
         <f>B28</f>
         <v/>
       </c>
-      <c r="C40" s="13">
+      <c r="C40" s="14">
         <f>C28</f>
         <v/>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="22">
         <f>N28</f>
         <v/>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="15">
         <f>IF(D40&gt;=20, 7.5, IF(D40&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F40" s="22">
+      <c r="F40" s="23">
         <f>ROUND(MAX(D40-E40, 0), 2)</f>
         <v/>
       </c>
-      <c r="G40" s="22">
+      <c r="G40" s="23">
         <f>ROUND(D40+E40, 2)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="12">
+      <c r="B41" s="13">
         <f>B29</f>
         <v/>
       </c>
-      <c r="C41" s="13">
+      <c r="C41" s="14">
         <f>C29</f>
         <v/>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="22">
         <f>N29</f>
         <v/>
       </c>
-      <c r="E41" s="14">
+      <c r="E41" s="15">
         <f>IF(D41&gt;=20, 7.5, IF(D41&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="23">
         <f>ROUND(MAX(D41-E41, 0), 2)</f>
         <v/>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="23">
         <f>ROUND(D41+E41, 2)</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="2" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="13">
+        <f>B30</f>
+        <v/>
+      </c>
+      <c r="C42" s="14">
+        <f>C30</f>
+        <v/>
+      </c>
+      <c r="D42" s="22">
+        <f>N30</f>
+        <v/>
+      </c>
+      <c r="E42" s="15">
+        <f>IF(D42&gt;=20, 7.5, IF(D42&gt;=10, 5.0, 2.5))</f>
+        <v/>
+      </c>
+      <c r="F42" s="23">
+        <f>ROUND(MAX(D42-E42, 0), 2)</f>
+        <v/>
+      </c>
+      <c r="G42" s="23">
+        <f>ROUND(D42+E42, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Formula Reference</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="23" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>1. Signal_i = TAA 의견 → 수치 (SOW=+2, OW=+1, N=0, UW=-1, SUW=-2)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="23" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>2. Gap_i = SAA_i - Peer_i</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="23" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="24" t="inlineStr">
         <is>
           <t>3. Aligned = 1 if Signal×Gap ≥ 0, else 0</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="23" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="24" t="inlineStr">
         <is>
           <t>4. Damping_i = Aligned × (1 - d) + d    (d = Damping 파라미터)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="23" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="24" t="inlineStr">
         <is>
           <t>5. Tilt_i = |Gap_i| × Damping_i  (gap=0이면 Peer_i × Min Tilt Rate)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="23" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="24" t="inlineStr">
         <is>
           <t>6. Adj_i = α × Signal_i × Tilt_i</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="23" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="24" t="inlineStr">
         <is>
           <t>7. Raw_i = MAX( Peer_i + Adj_i,  1.0 )</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="23" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="24" t="inlineStr">
         <is>
           <t>8. Final_i = Raw_i / Σ Raw_j × 100</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="23" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="24" t="inlineStr">
         <is>
           <t>9. Range: Final ≥ 20% → ±7.5%p, ≥ 10% → ±5%p, &lt; 10% → ±2.5%p</t>
         </is>
@@ -1781,7 +1796,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F11 F12 F13 F14 F15 F16 F17 F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="잘못된 입력" error="TAA 옵션에서 선택하세요" type="list">
+    <dataValidation sqref="F12 F13 F14 F15 F16 F17 F18 F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="잘못된 입력" error="TAA 옵션에서 선택하세요" type="list">
       <formula1>"Strong OW,Overweight,Neutral,Underweight,Strong UW"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1795,11 +1810,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L51"/>
+  <dimension ref="B1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -1808,10 +1823,8 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1847,13 +1860,15 @@
           <t>← 0~1 (보수적 → 적극적)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Strong OW</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>2</v>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>TAA</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1870,13 +1885,13 @@
           <t>← 0=Peer중심, 1=SAA중심</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Overweight</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>1</v>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Strong OW</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1893,1010 +1908,1020 @@
           <t>← Base 대비 Tilt 비율</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Overweight</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I7" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="H7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I8" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="H8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Strong UW</t>
         </is>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I9" s="8" t="n">
         <v>-2</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Region Inputs</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="7" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>SAA(%)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Peer(%)</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>TAA</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E12" s="11" t="n">
         <v>45.5</v>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>유럽</t>
         </is>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <v>10.5</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E13" s="11" t="n">
         <v>12.6</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>일본</t>
         </is>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E14" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>중국</t>
         </is>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <v>2.1</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E15" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D16" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E16" s="11" t="n">
         <v>2.1</v>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>주식</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>기타</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <v>1.4</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E17" s="11" t="n">
         <v>2.8</v>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>채권</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>미국</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E18" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>채권</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>한국</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E19" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>SAA</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Peer</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Tilt</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Adj</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Raw</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Final(%)</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>vs Peer</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="12">
-        <f>B11</f>
-        <v/>
-      </c>
-      <c r="C22" s="13">
-        <f>C11</f>
-        <v/>
-      </c>
-      <c r="D22" s="14">
-        <f>D11</f>
-        <v/>
-      </c>
-      <c r="E22" s="14">
-        <f>E11</f>
-        <v/>
-      </c>
-      <c r="F22" s="15">
-        <f>IF(F11="Strong OW",2,IF(F11="Overweight",1,IF(F11="Neutral",0,IF(F11="Underweight",-1,IF(F11="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>$C$5*D22+(1-$C$5)*E22</f>
-        <v/>
-      </c>
-      <c r="H22" s="16">
-        <f>G22*$C$6</f>
-        <v/>
-      </c>
-      <c r="I22" s="17">
-        <f>$C$4*F22*H22</f>
-        <v/>
-      </c>
-      <c r="J22" s="16">
-        <f>MAX(G22+I22, 1.0)</f>
-        <v/>
-      </c>
-      <c r="K22" s="18">
-        <f>ROUND(J22/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L22" s="17">
-        <f>ROUND(K22-E22, 2)</f>
-        <v/>
-      </c>
-    </row>
     <row r="23">
-      <c r="B23" s="12">
+      <c r="B23" s="13">
         <f>B12</f>
         <v/>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="14">
         <f>C12</f>
         <v/>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="15">
         <f>D12</f>
         <v/>
       </c>
-      <c r="E23" s="14">
+      <c r="E23" s="15">
         <f>E12</f>
         <v/>
       </c>
-      <c r="F23" s="15">
-        <f>IF(F12="Strong OW",2,IF(F12="Overweight",1,IF(F12="Neutral",0,IF(F12="Underweight",-1,IF(F12="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
+      <c r="F23" s="16">
+        <f>VLOOKUP(F12,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G23" s="17">
         <f>$C$5*D23+(1-$C$5)*E23</f>
         <v/>
       </c>
-      <c r="H23" s="16">
+      <c r="H23" s="17">
         <f>G23*$C$6</f>
         <v/>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="18">
         <f>$C$4*F23*H23</f>
         <v/>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="17">
         <f>MAX(G23+I23, 1.0)</f>
         <v/>
       </c>
-      <c r="K23" s="18">
-        <f>ROUND(J23/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L23" s="17">
+      <c r="K23" s="19">
+        <f>ROUND(J23/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
         <f>ROUND(K23-E23, 2)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="12">
+      <c r="B24" s="13">
         <f>B13</f>
         <v/>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="14">
         <f>C13</f>
         <v/>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="15">
         <f>D13</f>
         <v/>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="15">
         <f>E13</f>
         <v/>
       </c>
-      <c r="F24" s="15">
-        <f>IF(F13="Strong OW",2,IF(F13="Overweight",1,IF(F13="Neutral",0,IF(F13="Underweight",-1,IF(F13="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
+      <c r="F24" s="16">
+        <f>VLOOKUP(F13,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G24" s="17">
         <f>$C$5*D24+(1-$C$5)*E24</f>
         <v/>
       </c>
-      <c r="H24" s="16">
+      <c r="H24" s="17">
         <f>G24*$C$6</f>
         <v/>
       </c>
-      <c r="I24" s="17">
+      <c r="I24" s="18">
         <f>$C$4*F24*H24</f>
         <v/>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="17">
         <f>MAX(G24+I24, 1.0)</f>
         <v/>
       </c>
-      <c r="K24" s="18">
-        <f>ROUND(J24/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L24" s="17">
+      <c r="K24" s="19">
+        <f>ROUND(J24/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L24" s="18">
         <f>ROUND(K24-E24, 2)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="12">
+      <c r="B25" s="13">
         <f>B14</f>
         <v/>
       </c>
-      <c r="C25" s="13">
+      <c r="C25" s="14">
         <f>C14</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="15">
         <f>D14</f>
         <v/>
       </c>
-      <c r="E25" s="14">
+      <c r="E25" s="15">
         <f>E14</f>
         <v/>
       </c>
-      <c r="F25" s="15">
-        <f>IF(F14="Strong OW",2,IF(F14="Overweight",1,IF(F14="Neutral",0,IF(F14="Underweight",-1,IF(F14="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
+      <c r="F25" s="16">
+        <f>VLOOKUP(F14,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G25" s="17">
         <f>$C$5*D25+(1-$C$5)*E25</f>
         <v/>
       </c>
-      <c r="H25" s="16">
+      <c r="H25" s="17">
         <f>G25*$C$6</f>
         <v/>
       </c>
-      <c r="I25" s="17">
+      <c r="I25" s="18">
         <f>$C$4*F25*H25</f>
         <v/>
       </c>
-      <c r="J25" s="16">
+      <c r="J25" s="17">
         <f>MAX(G25+I25, 1.0)</f>
         <v/>
       </c>
-      <c r="K25" s="18">
-        <f>ROUND(J25/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L25" s="17">
+      <c r="K25" s="19">
+        <f>ROUND(J25/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
         <f>ROUND(K25-E25, 2)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="12">
+      <c r="B26" s="13">
         <f>B15</f>
         <v/>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="14">
         <f>C15</f>
         <v/>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="15">
         <f>D15</f>
         <v/>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="15">
         <f>E15</f>
         <v/>
       </c>
-      <c r="F26" s="15">
-        <f>IF(F15="Strong OW",2,IF(F15="Overweight",1,IF(F15="Neutral",0,IF(F15="Underweight",-1,IF(F15="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
+      <c r="F26" s="16">
+        <f>VLOOKUP(F15,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G26" s="17">
         <f>$C$5*D26+(1-$C$5)*E26</f>
         <v/>
       </c>
-      <c r="H26" s="16">
+      <c r="H26" s="17">
         <f>G26*$C$6</f>
         <v/>
       </c>
-      <c r="I26" s="17">
+      <c r="I26" s="18">
         <f>$C$4*F26*H26</f>
         <v/>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="17">
         <f>MAX(G26+I26, 1.0)</f>
         <v/>
       </c>
-      <c r="K26" s="18">
-        <f>ROUND(J26/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L26" s="17">
+      <c r="K26" s="19">
+        <f>ROUND(J26/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
         <f>ROUND(K26-E26, 2)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="12">
+      <c r="B27" s="13">
         <f>B16</f>
         <v/>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="14">
         <f>C16</f>
         <v/>
       </c>
-      <c r="D27" s="14">
+      <c r="D27" s="15">
         <f>D16</f>
         <v/>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="15">
         <f>E16</f>
         <v/>
       </c>
-      <c r="F27" s="15">
-        <f>IF(F16="Strong OW",2,IF(F16="Overweight",1,IF(F16="Neutral",0,IF(F16="Underweight",-1,IF(F16="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
+      <c r="F27" s="16">
+        <f>VLOOKUP(F16,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G27" s="17">
         <f>$C$5*D27+(1-$C$5)*E27</f>
         <v/>
       </c>
-      <c r="H27" s="16">
+      <c r="H27" s="17">
         <f>G27*$C$6</f>
         <v/>
       </c>
-      <c r="I27" s="17">
+      <c r="I27" s="18">
         <f>$C$4*F27*H27</f>
         <v/>
       </c>
-      <c r="J27" s="16">
+      <c r="J27" s="17">
         <f>MAX(G27+I27, 1.0)</f>
         <v/>
       </c>
-      <c r="K27" s="18">
-        <f>ROUND(J27/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L27" s="17">
+      <c r="K27" s="19">
+        <f>ROUND(J27/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
         <f>ROUND(K27-E27, 2)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="12">
+      <c r="B28" s="13">
         <f>B17</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>C17</f>
         <v/>
       </c>
-      <c r="D28" s="14">
+      <c r="D28" s="15">
         <f>D17</f>
         <v/>
       </c>
-      <c r="E28" s="14">
+      <c r="E28" s="15">
         <f>E17</f>
         <v/>
       </c>
-      <c r="F28" s="15">
-        <f>IF(F17="Strong OW",2,IF(F17="Overweight",1,IF(F17="Neutral",0,IF(F17="Underweight",-1,IF(F17="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
+      <c r="F28" s="16">
+        <f>VLOOKUP(F17,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G28" s="17">
         <f>$C$5*D28+(1-$C$5)*E28</f>
         <v/>
       </c>
-      <c r="H28" s="16">
+      <c r="H28" s="17">
         <f>G28*$C$6</f>
         <v/>
       </c>
-      <c r="I28" s="17">
+      <c r="I28" s="18">
         <f>$C$4*F28*H28</f>
         <v/>
       </c>
-      <c r="J28" s="16">
+      <c r="J28" s="17">
         <f>MAX(G28+I28, 1.0)</f>
         <v/>
       </c>
-      <c r="K28" s="18">
-        <f>ROUND(J28/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L28" s="17">
+      <c r="K28" s="19">
+        <f>ROUND(J28/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
         <f>ROUND(K28-E28, 2)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="12">
+      <c r="B29" s="13">
         <f>B18</f>
         <v/>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="14">
         <f>C18</f>
         <v/>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="15">
         <f>D18</f>
         <v/>
       </c>
-      <c r="E29" s="14">
+      <c r="E29" s="15">
         <f>E18</f>
         <v/>
       </c>
-      <c r="F29" s="15">
-        <f>IF(F18="Strong OW",2,IF(F18="Overweight",1,IF(F18="Neutral",0,IF(F18="Underweight",-1,IF(F18="Strong UW",-2,0)))))</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
+      <c r="F29" s="16">
+        <f>VLOOKUP(F18,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G29" s="17">
         <f>$C$5*D29+(1-$C$5)*E29</f>
         <v/>
       </c>
-      <c r="H29" s="16">
+      <c r="H29" s="17">
         <f>G29*$C$6</f>
         <v/>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="18">
         <f>$C$4*F29*H29</f>
         <v/>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="17">
         <f>MAX(G29+I29, 1.0)</f>
         <v/>
       </c>
-      <c r="K29" s="18">
-        <f>ROUND(J29/SUM(J22:J29)*100, 2)</f>
-        <v/>
-      </c>
-      <c r="L29" s="17">
+      <c r="K29" s="19">
+        <f>ROUND(J29/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L29" s="18">
         <f>ROUND(K29-E29, 2)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="19" t="inlineStr">
+      <c r="B30" s="13">
+        <f>B19</f>
+        <v/>
+      </c>
+      <c r="C30" s="14">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="F30" s="16">
+        <f>VLOOKUP(F19,$H$5:$I$9,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="G30" s="17">
+        <f>$C$5*D30+(1-$C$5)*E30</f>
+        <v/>
+      </c>
+      <c r="H30" s="17">
+        <f>G30*$C$6</f>
+        <v/>
+      </c>
+      <c r="I30" s="18">
+        <f>$C$4*F30*H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="17">
+        <f>MAX(G30+I30, 1.0)</f>
+        <v/>
+      </c>
+      <c r="K30" s="19">
+        <f>ROUND(J30/SUM(J23:J30)*100, 2)</f>
+        <v/>
+      </c>
+      <c r="L30" s="18">
+        <f>ROUND(K30-E30, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D30" s="20">
-        <f>SUM(D22:D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="20">
-        <f>SUM(E22:E29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="20">
-        <f>SUM(G22:G29)</f>
-        <v/>
-      </c>
-      <c r="J30" s="20">
-        <f>SUM(J22:J29)</f>
-        <v/>
-      </c>
-      <c r="K30" s="20">
-        <f>SUM(K22:K29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="2" t="inlineStr">
+      <c r="D31" s="21">
+        <f>SUM(D23:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="21">
+        <f>SUM(E23:E30)</f>
+        <v/>
+      </c>
+      <c r="G31" s="21">
+        <f>SUM(G23:G30)</f>
+        <v/>
+      </c>
+      <c r="J31" s="21">
+        <f>SUM(J23:J30)</f>
+        <v/>
+      </c>
+      <c r="K31" s="21">
+        <f>SUM(K23:K30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Range (허용 범위)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>자산</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>지역</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Final(%)</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Half Width</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Low(%)</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>High(%)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="12">
-        <f>B22</f>
-        <v/>
-      </c>
-      <c r="C34" s="13">
-        <f>C22</f>
-        <v/>
-      </c>
-      <c r="D34" s="21">
-        <f>K22</f>
-        <v/>
-      </c>
-      <c r="E34" s="14">
-        <f>IF(D34&gt;=20, 7.5, IF(D34&gt;=10, 5.0, 2.5))</f>
-        <v/>
-      </c>
-      <c r="F34" s="22">
-        <f>ROUND(MAX(D34-E34, 0), 2)</f>
-        <v/>
-      </c>
-      <c r="G34" s="22">
-        <f>ROUND(D34+E34, 2)</f>
-        <v/>
-      </c>
-    </row>
     <row r="35">
-      <c r="B35" s="12">
+      <c r="B35" s="13">
         <f>B23</f>
         <v/>
       </c>
-      <c r="C35" s="13">
+      <c r="C35" s="14">
         <f>C23</f>
         <v/>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="22">
         <f>K23</f>
         <v/>
       </c>
-      <c r="E35" s="14">
+      <c r="E35" s="15">
         <f>IF(D35&gt;=20, 7.5, IF(D35&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F35" s="22">
+      <c r="F35" s="23">
         <f>ROUND(MAX(D35-E35, 0), 2)</f>
         <v/>
       </c>
-      <c r="G35" s="22">
+      <c r="G35" s="23">
         <f>ROUND(D35+E35, 2)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="12">
+      <c r="B36" s="13">
         <f>B24</f>
         <v/>
       </c>
-      <c r="C36" s="13">
+      <c r="C36" s="14">
         <f>C24</f>
         <v/>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="22">
         <f>K24</f>
         <v/>
       </c>
-      <c r="E36" s="14">
+      <c r="E36" s="15">
         <f>IF(D36&gt;=20, 7.5, IF(D36&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F36" s="22">
+      <c r="F36" s="23">
         <f>ROUND(MAX(D36-E36, 0), 2)</f>
         <v/>
       </c>
-      <c r="G36" s="22">
+      <c r="G36" s="23">
         <f>ROUND(D36+E36, 2)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="12">
+      <c r="B37" s="13">
         <f>B25</f>
         <v/>
       </c>
-      <c r="C37" s="13">
+      <c r="C37" s="14">
         <f>C25</f>
         <v/>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="22">
         <f>K25</f>
         <v/>
       </c>
-      <c r="E37" s="14">
+      <c r="E37" s="15">
         <f>IF(D37&gt;=20, 7.5, IF(D37&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="23">
         <f>ROUND(MAX(D37-E37, 0), 2)</f>
         <v/>
       </c>
-      <c r="G37" s="22">
+      <c r="G37" s="23">
         <f>ROUND(D37+E37, 2)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="12">
+      <c r="B38" s="13">
         <f>B26</f>
         <v/>
       </c>
-      <c r="C38" s="13">
+      <c r="C38" s="14">
         <f>C26</f>
         <v/>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="22">
         <f>K26</f>
         <v/>
       </c>
-      <c r="E38" s="14">
+      <c r="E38" s="15">
         <f>IF(D38&gt;=20, 7.5, IF(D38&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F38" s="22">
+      <c r="F38" s="23">
         <f>ROUND(MAX(D38-E38, 0), 2)</f>
         <v/>
       </c>
-      <c r="G38" s="22">
+      <c r="G38" s="23">
         <f>ROUND(D38+E38, 2)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="12">
+      <c r="B39" s="13">
         <f>B27</f>
         <v/>
       </c>
-      <c r="C39" s="13">
+      <c r="C39" s="14">
         <f>C27</f>
         <v/>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="22">
         <f>K27</f>
         <v/>
       </c>
-      <c r="E39" s="14">
+      <c r="E39" s="15">
         <f>IF(D39&gt;=20, 7.5, IF(D39&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="23">
         <f>ROUND(MAX(D39-E39, 0), 2)</f>
         <v/>
       </c>
-      <c r="G39" s="22">
+      <c r="G39" s="23">
         <f>ROUND(D39+E39, 2)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="12">
+      <c r="B40" s="13">
         <f>B28</f>
         <v/>
       </c>
-      <c r="C40" s="13">
+      <c r="C40" s="14">
         <f>C28</f>
         <v/>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="22">
         <f>K28</f>
         <v/>
       </c>
-      <c r="E40" s="14">
+      <c r="E40" s="15">
         <f>IF(D40&gt;=20, 7.5, IF(D40&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F40" s="22">
+      <c r="F40" s="23">
         <f>ROUND(MAX(D40-E40, 0), 2)</f>
         <v/>
       </c>
-      <c r="G40" s="22">
+      <c r="G40" s="23">
         <f>ROUND(D40+E40, 2)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="12">
+      <c r="B41" s="13">
         <f>B29</f>
         <v/>
       </c>
-      <c r="C41" s="13">
+      <c r="C41" s="14">
         <f>C29</f>
         <v/>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="22">
         <f>K29</f>
         <v/>
       </c>
-      <c r="E41" s="14">
+      <c r="E41" s="15">
         <f>IF(D41&gt;=20, 7.5, IF(D41&gt;=10, 5.0, 2.5))</f>
         <v/>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="23">
         <f>ROUND(MAX(D41-E41, 0), 2)</f>
         <v/>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="23">
         <f>ROUND(D41+E41, 2)</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="2" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="13">
+        <f>B30</f>
+        <v/>
+      </c>
+      <c r="C42" s="14">
+        <f>C30</f>
+        <v/>
+      </c>
+      <c r="D42" s="22">
+        <f>K30</f>
+        <v/>
+      </c>
+      <c r="E42" s="15">
+        <f>IF(D42&gt;=20, 7.5, IF(D42&gt;=10, 5.0, 2.5))</f>
+        <v/>
+      </c>
+      <c r="F42" s="23">
+        <f>ROUND(MAX(D42-E42, 0), 2)</f>
+        <v/>
+      </c>
+      <c r="G42" s="23">
+        <f>ROUND(D42+E42, 2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Formula Reference</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="23" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>1. Signal_i = TAA 의견 → 수치 (SOW=+2, OW=+1, N=0, UW=-1, SUW=-2)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="23" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>2. Base_i = w × SAA_i + (1-w) × Peer_i</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="23" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="24" t="inlineStr">
         <is>
           <t>3. Tilt_i = Base_i × Tilt Rate</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="23" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="24" t="inlineStr">
         <is>
           <t>4. Adj_i = α × Signal_i × Tilt_i</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="23" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="24" t="inlineStr">
         <is>
           <t>5. Raw_i = MAX( Base_i + Adj_i,  1.0 )</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="23" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="24" t="inlineStr">
         <is>
           <t>6. Final_i = Raw_i / Σ Raw_j × 100</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="23" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="24" t="inlineStr">
         <is>
           <t>7. Range: Final ≥ 20% → ±7.5%p, ≥ 10% → ±5%p, &lt; 10% → ±2.5%p</t>
         </is>
@@ -2907,7 +2932,7 @@
     <mergeCell ref="B1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F11 F12 F13 F14 F15 F16 F17 F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F12 F13 F14 F15 F16 F17 F18 F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Strong OW,Overweight,Neutral,Underweight,Strong UW"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add vs SAA and vintage propagation to Excel
</commit_message>
<xml_diff>
--- a/TAA_Dashboard.xlsx
+++ b/TAA_Dashboard.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O54"/>
+  <dimension ref="B1:P91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -568,6 +568,7 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -986,6 +987,11 @@
           <t>vs Peer</t>
         </is>
       </c>
+      <c r="P22" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="13">
@@ -1044,6 +1050,10 @@
         <f>ROUND(N23-E23, 2)</f>
         <v/>
       </c>
+      <c r="P23" s="18">
+        <f>ROUND(N23-D23, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="13">
@@ -1102,6 +1112,10 @@
         <f>ROUND(N24-E24, 2)</f>
         <v/>
       </c>
+      <c r="P24" s="18">
+        <f>ROUND(N24-D24, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="13">
@@ -1160,6 +1174,10 @@
         <f>ROUND(N25-E25, 2)</f>
         <v/>
       </c>
+      <c r="P25" s="18">
+        <f>ROUND(N25-D25, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="13">
@@ -1218,6 +1236,10 @@
         <f>ROUND(N26-E26, 2)</f>
         <v/>
       </c>
+      <c r="P26" s="18">
+        <f>ROUND(N26-D26, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="13">
@@ -1276,6 +1298,10 @@
         <f>ROUND(N27-E27, 2)</f>
         <v/>
       </c>
+      <c r="P27" s="18">
+        <f>ROUND(N27-D27, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="13">
@@ -1334,6 +1360,10 @@
         <f>ROUND(N28-E28, 2)</f>
         <v/>
       </c>
+      <c r="P28" s="18">
+        <f>ROUND(N28-D28, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="13">
@@ -1392,6 +1422,10 @@
         <f>ROUND(N29-E29, 2)</f>
         <v/>
       </c>
+      <c r="P29" s="18">
+        <f>ROUND(N29-D29, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="13">
@@ -1450,6 +1484,10 @@
         <f>ROUND(N30-E30, 2)</f>
         <v/>
       </c>
+      <c r="P30" s="18">
+        <f>ROUND(N30-D30, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="20" t="inlineStr">
@@ -1789,6 +1827,1149 @@
         <is>
           <t>9. Range: Final ≥ 20% → ±7.5%p, ≥ 10% → ±5%p, &lt; 10% → ±2.5%p</t>
         </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2030  (주식 40% / 채권 60%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="E59" s="18">
+        <f>IF(D23&gt;=0.5,(M23-D23)/D23,M23-D23)</f>
+        <v/>
+      </c>
+      <c r="F59" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D59*(1+E59),D59+E59),1.0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="19">
+        <f>ROUND(F59/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H59" s="18">
+        <f>ROUND(G59-D59,2)</f>
+        <v/>
+      </c>
+      <c r="I59" s="17">
+        <f>ROUND(MAX(G59-IF(G59&gt;=20,7.5,IF(G59&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J59" s="17">
+        <f>ROUND(G59+IF(G59&gt;=20,7.5,IF(G59&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" s="18">
+        <f>IF(D24&gt;=0.5,(M24-D24)/D24,M24-D24)</f>
+        <v/>
+      </c>
+      <c r="F60" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D60*(1+E60),D60+E60),1.0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="19">
+        <f>ROUND(F60/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H60" s="18">
+        <f>ROUND(G60-D60,2)</f>
+        <v/>
+      </c>
+      <c r="I60" s="17">
+        <f>ROUND(MAX(G60-IF(G60&gt;=20,7.5,IF(G60&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J60" s="17">
+        <f>ROUND(G60+IF(G60&gt;=20,7.5,IF(G60&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="18">
+        <f>IF(D25&gt;=0.5,(M25-D25)/D25,M25-D25)</f>
+        <v/>
+      </c>
+      <c r="F61" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D61*(1+E61),D61+E61),1.0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="19">
+        <f>ROUND(F61/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H61" s="18">
+        <f>ROUND(G61-D61,2)</f>
+        <v/>
+      </c>
+      <c r="I61" s="17">
+        <f>ROUND(MAX(G61-IF(G61&gt;=20,7.5,IF(G61&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J61" s="17">
+        <f>ROUND(G61+IF(G61&gt;=20,7.5,IF(G61&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E62" s="18">
+        <f>IF(D26&gt;=0.5,(M26-D26)/D26,M26-D26)</f>
+        <v/>
+      </c>
+      <c r="F62" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D62*(1+E62),D62+E62),1.0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="19">
+        <f>ROUND(F62/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H62" s="18">
+        <f>ROUND(G62-D62,2)</f>
+        <v/>
+      </c>
+      <c r="I62" s="17">
+        <f>ROUND(MAX(G62-IF(G62&gt;=20,7.5,IF(G62&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J62" s="17">
+        <f>ROUND(G62+IF(G62&gt;=20,7.5,IF(G62&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="18">
+        <f>IF(D27&gt;=0.5,(M27-D27)/D27,M27-D27)</f>
+        <v/>
+      </c>
+      <c r="F63" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D63*(1+E63),D63+E63),1.0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="19">
+        <f>ROUND(F63/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H63" s="18">
+        <f>ROUND(G63-D63,2)</f>
+        <v/>
+      </c>
+      <c r="I63" s="17">
+        <f>ROUND(MAX(G63-IF(G63&gt;=20,7.5,IF(G63&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J63" s="17">
+        <f>ROUND(G63+IF(G63&gt;=20,7.5,IF(G63&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E64" s="18">
+        <f>IF(D28&gt;=0.5,(M28-D28)/D28,M28-D28)</f>
+        <v/>
+      </c>
+      <c r="F64" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D64*(1+E64),D64+E64),1.0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="19">
+        <f>ROUND(F64/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H64" s="18">
+        <f>ROUND(G64-D64,2)</f>
+        <v/>
+      </c>
+      <c r="I64" s="17">
+        <f>ROUND(MAX(G64-IF(G64&gt;=20,7.5,IF(G64&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J64" s="17">
+        <f>ROUND(G64+IF(G64&gt;=20,7.5,IF(G64&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D65" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="E65" s="18">
+        <f>IF(D29&gt;=0.5,(M29-D29)/D29,M29-D29)</f>
+        <v/>
+      </c>
+      <c r="F65" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D65*(1+E65),D65+E65),1.0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="19">
+        <f>ROUND(F65/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H65" s="18">
+        <f>ROUND(G65-D65,2)</f>
+        <v/>
+      </c>
+      <c r="I65" s="17">
+        <f>ROUND(MAX(G65-IF(G65&gt;=20,7.5,IF(G65&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J65" s="17">
+        <f>ROUND(G65+IF(G65&gt;=20,7.5,IF(G65&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D66" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="E66" s="18">
+        <f>IF(D30&gt;=0.5,(M30-D30)/D30,M30-D30)</f>
+        <v/>
+      </c>
+      <c r="F66" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D66*(1+E66),D66+E66),1.0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="19">
+        <f>ROUND(F66/SUM(F59:F66)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H66" s="18">
+        <f>ROUND(G66-D66,2)</f>
+        <v/>
+      </c>
+      <c r="I66" s="17">
+        <f>ROUND(MAX(G66-IF(G66&gt;=20,7.5,IF(G66&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J66" s="17">
+        <f>ROUND(G66+IF(G66&gt;=20,7.5,IF(G66&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D67" s="21">
+        <f>SUM(D59:D66)</f>
+        <v/>
+      </c>
+      <c r="G67" s="21">
+        <f>SUM(G59:G66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2040  (주식 55% / 채권 45%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D71" s="17" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="E71" s="18">
+        <f>IF(D23&gt;=0.5,(M23-D23)/D23,M23-D23)</f>
+        <v/>
+      </c>
+      <c r="F71" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D71*(1+E71),D71+E71),1.0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="19">
+        <f>ROUND(F71/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H71" s="18">
+        <f>ROUND(G71-D71,2)</f>
+        <v/>
+      </c>
+      <c r="I71" s="17">
+        <f>ROUND(MAX(G71-IF(G71&gt;=20,7.5,IF(G71&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J71" s="17">
+        <f>ROUND(G71+IF(G71&gt;=20,7.5,IF(G71&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D72" s="17" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="E72" s="18">
+        <f>IF(D24&gt;=0.5,(M24-D24)/D24,M24-D24)</f>
+        <v/>
+      </c>
+      <c r="F72" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D72*(1+E72),D72+E72),1.0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="19">
+        <f>ROUND(F72/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H72" s="18">
+        <f>ROUND(G72-D72,2)</f>
+        <v/>
+      </c>
+      <c r="I72" s="17">
+        <f>ROUND(MAX(G72-IF(G72&gt;=20,7.5,IF(G72&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J72" s="17">
+        <f>ROUND(G72+IF(G72&gt;=20,7.5,IF(G72&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E73" s="18">
+        <f>IF(D25&gt;=0.5,(M25-D25)/D25,M25-D25)</f>
+        <v/>
+      </c>
+      <c r="F73" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D73*(1+E73),D73+E73),1.0)</f>
+        <v/>
+      </c>
+      <c r="G73" s="19">
+        <f>ROUND(F73/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H73" s="18">
+        <f>ROUND(G73-D73,2)</f>
+        <v/>
+      </c>
+      <c r="I73" s="17">
+        <f>ROUND(MAX(G73-IF(G73&gt;=20,7.5,IF(G73&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J73" s="17">
+        <f>ROUND(G73+IF(G73&gt;=20,7.5,IF(G73&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E74" s="18">
+        <f>IF(D26&gt;=0.5,(M26-D26)/D26,M26-D26)</f>
+        <v/>
+      </c>
+      <c r="F74" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D74*(1+E74),D74+E74),1.0)</f>
+        <v/>
+      </c>
+      <c r="G74" s="19">
+        <f>ROUND(F74/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H74" s="18">
+        <f>ROUND(G74-D74,2)</f>
+        <v/>
+      </c>
+      <c r="I74" s="17">
+        <f>ROUND(MAX(G74-IF(G74&gt;=20,7.5,IF(G74&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J74" s="17">
+        <f>ROUND(G74+IF(G74&gt;=20,7.5,IF(G74&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D75" s="17" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E75" s="18">
+        <f>IF(D27&gt;=0.5,(M27-D27)/D27,M27-D27)</f>
+        <v/>
+      </c>
+      <c r="F75" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D75*(1+E75),D75+E75),1.0)</f>
+        <v/>
+      </c>
+      <c r="G75" s="19">
+        <f>ROUND(F75/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H75" s="18">
+        <f>ROUND(G75-D75,2)</f>
+        <v/>
+      </c>
+      <c r="I75" s="17">
+        <f>ROUND(MAX(G75-IF(G75&gt;=20,7.5,IF(G75&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J75" s="17">
+        <f>ROUND(G75+IF(G75&gt;=20,7.5,IF(G75&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="18">
+        <f>IF(D28&gt;=0.5,(M28-D28)/D28,M28-D28)</f>
+        <v/>
+      </c>
+      <c r="F76" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D76*(1+E76),D76+E76),1.0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="19">
+        <f>ROUND(F76/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H76" s="18">
+        <f>ROUND(G76-D76,2)</f>
+        <v/>
+      </c>
+      <c r="I76" s="17">
+        <f>ROUND(MAX(G76-IF(G76&gt;=20,7.5,IF(G76&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J76" s="17">
+        <f>ROUND(G76+IF(G76&gt;=20,7.5,IF(G76&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D77" s="17" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E77" s="18">
+        <f>IF(D29&gt;=0.5,(M29-D29)/D29,M29-D29)</f>
+        <v/>
+      </c>
+      <c r="F77" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D77*(1+E77),D77+E77),1.0)</f>
+        <v/>
+      </c>
+      <c r="G77" s="19">
+        <f>ROUND(F77/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H77" s="18">
+        <f>ROUND(G77-D77,2)</f>
+        <v/>
+      </c>
+      <c r="I77" s="17">
+        <f>ROUND(MAX(G77-IF(G77&gt;=20,7.5,IF(G77&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J77" s="17">
+        <f>ROUND(G77+IF(G77&gt;=20,7.5,IF(G77&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D78" s="17" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E78" s="18">
+        <f>IF(D30&gt;=0.5,(M30-D30)/D30,M30-D30)</f>
+        <v/>
+      </c>
+      <c r="F78" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D78*(1+E78),D78+E78),1.0)</f>
+        <v/>
+      </c>
+      <c r="G78" s="19">
+        <f>ROUND(F78/SUM(F71:F78)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H78" s="18">
+        <f>ROUND(G78-D78,2)</f>
+        <v/>
+      </c>
+      <c r="I78" s="17">
+        <f>ROUND(MAX(G78-IF(G78&gt;=20,7.5,IF(G78&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J78" s="17">
+        <f>ROUND(G78+IF(G78&gt;=20,7.5,IF(G78&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D79" s="21">
+        <f>SUM(D71:D78)</f>
+        <v/>
+      </c>
+      <c r="G79" s="21">
+        <f>SUM(G71:G78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2060  (주식 90% / 채권 10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D83" s="17" t="n">
+        <v>63</v>
+      </c>
+      <c r="E83" s="18">
+        <f>IF(D23&gt;=0.5,(M23-D23)/D23,M23-D23)</f>
+        <v/>
+      </c>
+      <c r="F83" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D83*(1+E83),D83+E83),1.0)</f>
+        <v/>
+      </c>
+      <c r="G83" s="19">
+        <f>ROUND(F83/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H83" s="18">
+        <f>ROUND(G83-D83,2)</f>
+        <v/>
+      </c>
+      <c r="I83" s="17">
+        <f>ROUND(MAX(G83-IF(G83&gt;=20,7.5,IF(G83&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J83" s="17">
+        <f>ROUND(G83+IF(G83&gt;=20,7.5,IF(G83&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E84" s="18">
+        <f>IF(D24&gt;=0.5,(M24-D24)/D24,M24-D24)</f>
+        <v/>
+      </c>
+      <c r="F84" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D84*(1+E84),D84+E84),1.0)</f>
+        <v/>
+      </c>
+      <c r="G84" s="19">
+        <f>ROUND(F84/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H84" s="18">
+        <f>ROUND(G84-D84,2)</f>
+        <v/>
+      </c>
+      <c r="I84" s="17">
+        <f>ROUND(MAX(G84-IF(G84&gt;=20,7.5,IF(G84&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J84" s="17">
+        <f>ROUND(G84+IF(G84&gt;=20,7.5,IF(G84&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E85" s="18">
+        <f>IF(D25&gt;=0.5,(M25-D25)/D25,M25-D25)</f>
+        <v/>
+      </c>
+      <c r="F85" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D85*(1+E85),D85+E85),1.0)</f>
+        <v/>
+      </c>
+      <c r="G85" s="19">
+        <f>ROUND(F85/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H85" s="18">
+        <f>ROUND(G85-D85,2)</f>
+        <v/>
+      </c>
+      <c r="I85" s="17">
+        <f>ROUND(MAX(G85-IF(G85&gt;=20,7.5,IF(G85&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J85" s="17">
+        <f>ROUND(G85+IF(G85&gt;=20,7.5,IF(G85&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E86" s="18">
+        <f>IF(D26&gt;=0.5,(M26-D26)/D26,M26-D26)</f>
+        <v/>
+      </c>
+      <c r="F86" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D86*(1+E86),D86+E86),1.0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="19">
+        <f>ROUND(F86/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H86" s="18">
+        <f>ROUND(G86-D86,2)</f>
+        <v/>
+      </c>
+      <c r="I86" s="17">
+        <f>ROUND(MAX(G86-IF(G86&gt;=20,7.5,IF(G86&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J86" s="17">
+        <f>ROUND(G86+IF(G86&gt;=20,7.5,IF(G86&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D87" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E87" s="18">
+        <f>IF(D27&gt;=0.5,(M27-D27)/D27,M27-D27)</f>
+        <v/>
+      </c>
+      <c r="F87" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D87*(1+E87),D87+E87),1.0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="19">
+        <f>ROUND(F87/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H87" s="18">
+        <f>ROUND(G87-D87,2)</f>
+        <v/>
+      </c>
+      <c r="I87" s="17">
+        <f>ROUND(MAX(G87-IF(G87&gt;=20,7.5,IF(G87&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J87" s="17">
+        <f>ROUND(G87+IF(G87&gt;=20,7.5,IF(G87&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E88" s="18">
+        <f>IF(D28&gt;=0.5,(M28-D28)/D28,M28-D28)</f>
+        <v/>
+      </c>
+      <c r="F88" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D88*(1+E88),D88+E88),1.0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="19">
+        <f>ROUND(F88/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H88" s="18">
+        <f>ROUND(G88-D88,2)</f>
+        <v/>
+      </c>
+      <c r="I88" s="17">
+        <f>ROUND(MAX(G88-IF(G88&gt;=20,7.5,IF(G88&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J88" s="17">
+        <f>ROUND(G88+IF(G88&gt;=20,7.5,IF(G88&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D89" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E89" s="18">
+        <f>IF(D29&gt;=0.5,(M29-D29)/D29,M29-D29)</f>
+        <v/>
+      </c>
+      <c r="F89" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D89*(1+E89),D89+E89),1.0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="19">
+        <f>ROUND(F89/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H89" s="18">
+        <f>ROUND(G89-D89,2)</f>
+        <v/>
+      </c>
+      <c r="I89" s="17">
+        <f>ROUND(MAX(G89-IF(G89&gt;=20,7.5,IF(G89&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J89" s="17">
+        <f>ROUND(G89+IF(G89&gt;=20,7.5,IF(G89&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D90" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E90" s="18">
+        <f>IF(D30&gt;=0.5,(M30-D30)/D30,M30-D30)</f>
+        <v/>
+      </c>
+      <c r="F90" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D90*(1+E90),D90+E90),1.0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="19">
+        <f>ROUND(F90/SUM(F83:F90)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H90" s="18">
+        <f>ROUND(G90-D90,2)</f>
+        <v/>
+      </c>
+      <c r="I90" s="17">
+        <f>ROUND(MAX(G90-IF(G90&gt;=20,7.5,IF(G90&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J90" s="17">
+        <f>ROUND(G90+IF(G90&gt;=20,7.5,IF(G90&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D91" s="21">
+        <f>SUM(D83:D90)</f>
+        <v/>
+      </c>
+      <c r="G91" s="21">
+        <f>SUM(G83:G90)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1810,7 +2991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L52"/>
+  <dimension ref="B1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1825,6 +3006,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2228,6 +3410,11 @@
           <t>vs Peer</t>
         </is>
       </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="13">
@@ -2274,6 +3461,10 @@
         <f>ROUND(K23-E23, 2)</f>
         <v/>
       </c>
+      <c r="M23" s="18">
+        <f>ROUND(K23-D23, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="13">
@@ -2320,6 +3511,10 @@
         <f>ROUND(K24-E24, 2)</f>
         <v/>
       </c>
+      <c r="M24" s="18">
+        <f>ROUND(K24-D24, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="13">
@@ -2366,6 +3561,10 @@
         <f>ROUND(K25-E25, 2)</f>
         <v/>
       </c>
+      <c r="M25" s="18">
+        <f>ROUND(K25-D25, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="13">
@@ -2412,6 +3611,10 @@
         <f>ROUND(K26-E26, 2)</f>
         <v/>
       </c>
+      <c r="M26" s="18">
+        <f>ROUND(K26-D26, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="13">
@@ -2458,6 +3661,10 @@
         <f>ROUND(K27-E27, 2)</f>
         <v/>
       </c>
+      <c r="M27" s="18">
+        <f>ROUND(K27-D27, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="13">
@@ -2504,6 +3711,10 @@
         <f>ROUND(K28-E28, 2)</f>
         <v/>
       </c>
+      <c r="M28" s="18">
+        <f>ROUND(K28-D28, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="13">
@@ -2550,6 +3761,10 @@
         <f>ROUND(K29-E29, 2)</f>
         <v/>
       </c>
+      <c r="M29" s="18">
+        <f>ROUND(K29-D29, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="13">
@@ -2596,6 +3811,10 @@
         <f>ROUND(K30-E30, 2)</f>
         <v/>
       </c>
+      <c r="M30" s="18">
+        <f>ROUND(K30-D30, 2)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="20" t="inlineStr">
@@ -2925,6 +4144,1149 @@
         <is>
           <t>7. Range: Final ≥ 20% → ±7.5%p, ≥ 10% → ±5%p, &lt; 10% → ±2.5%p</t>
         </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2030  (주식 40% / 채권 60%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="E57" s="18">
+        <f>IF(D23&gt;=0.5,(J23-D23)/D23,J23-D23)</f>
+        <v/>
+      </c>
+      <c r="F57" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D57*(1+E57),D57+E57),1.0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="19">
+        <f>ROUND(F57/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H57" s="18">
+        <f>ROUND(G57-D57,2)</f>
+        <v/>
+      </c>
+      <c r="I57" s="17">
+        <f>ROUND(MAX(G57-IF(G57&gt;=20,7.5,IF(G57&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J57" s="17">
+        <f>ROUND(G57+IF(G57&gt;=20,7.5,IF(G57&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E58" s="18">
+        <f>IF(D24&gt;=0.5,(J24-D24)/D24,J24-D24)</f>
+        <v/>
+      </c>
+      <c r="F58" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D58*(1+E58),D58+E58),1.0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="19">
+        <f>ROUND(F58/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H58" s="18">
+        <f>ROUND(G58-D58,2)</f>
+        <v/>
+      </c>
+      <c r="I58" s="17">
+        <f>ROUND(MAX(G58-IF(G58&gt;=20,7.5,IF(G58&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J58" s="17">
+        <f>ROUND(G58+IF(G58&gt;=20,7.5,IF(G58&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" s="18">
+        <f>IF(D25&gt;=0.5,(J25-D25)/D25,J25-D25)</f>
+        <v/>
+      </c>
+      <c r="F59" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D59*(1+E59),D59+E59),1.0)</f>
+        <v/>
+      </c>
+      <c r="G59" s="19">
+        <f>ROUND(F59/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H59" s="18">
+        <f>ROUND(G59-D59,2)</f>
+        <v/>
+      </c>
+      <c r="I59" s="17">
+        <f>ROUND(MAX(G59-IF(G59&gt;=20,7.5,IF(G59&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J59" s="17">
+        <f>ROUND(G59+IF(G59&gt;=20,7.5,IF(G59&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E60" s="18">
+        <f>IF(D26&gt;=0.5,(J26-D26)/D26,J26-D26)</f>
+        <v/>
+      </c>
+      <c r="F60" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D60*(1+E60),D60+E60),1.0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="19">
+        <f>ROUND(F60/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H60" s="18">
+        <f>ROUND(G60-D60,2)</f>
+        <v/>
+      </c>
+      <c r="I60" s="17">
+        <f>ROUND(MAX(G60-IF(G60&gt;=20,7.5,IF(G60&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J60" s="17">
+        <f>ROUND(G60+IF(G60&gt;=20,7.5,IF(G60&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="18">
+        <f>IF(D27&gt;=0.5,(J27-D27)/D27,J27-D27)</f>
+        <v/>
+      </c>
+      <c r="F61" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D61*(1+E61),D61+E61),1.0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="19">
+        <f>ROUND(F61/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H61" s="18">
+        <f>ROUND(G61-D61,2)</f>
+        <v/>
+      </c>
+      <c r="I61" s="17">
+        <f>ROUND(MAX(G61-IF(G61&gt;=20,7.5,IF(G61&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J61" s="17">
+        <f>ROUND(G61+IF(G61&gt;=20,7.5,IF(G61&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E62" s="18">
+        <f>IF(D28&gt;=0.5,(J28-D28)/D28,J28-D28)</f>
+        <v/>
+      </c>
+      <c r="F62" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D62*(1+E62),D62+E62),1.0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="19">
+        <f>ROUND(F62/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H62" s="18">
+        <f>ROUND(G62-D62,2)</f>
+        <v/>
+      </c>
+      <c r="I62" s="17">
+        <f>ROUND(MAX(G62-IF(G62&gt;=20,7.5,IF(G62&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J62" s="17">
+        <f>ROUND(G62+IF(G62&gt;=20,7.5,IF(G62&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="E63" s="18">
+        <f>IF(D29&gt;=0.5,(J29-D29)/D29,J29-D29)</f>
+        <v/>
+      </c>
+      <c r="F63" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D63*(1+E63),D63+E63),1.0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="19">
+        <f>ROUND(F63/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H63" s="18">
+        <f>ROUND(G63-D63,2)</f>
+        <v/>
+      </c>
+      <c r="I63" s="17">
+        <f>ROUND(MAX(G63-IF(G63&gt;=20,7.5,IF(G63&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J63" s="17">
+        <f>ROUND(G63+IF(G63&gt;=20,7.5,IF(G63&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="E64" s="18">
+        <f>IF(D30&gt;=0.5,(J30-D30)/D30,J30-D30)</f>
+        <v/>
+      </c>
+      <c r="F64" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D64*(1+E64),D64+E64),1.0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="19">
+        <f>ROUND(F64/SUM(F57:F64)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H64" s="18">
+        <f>ROUND(G64-D64,2)</f>
+        <v/>
+      </c>
+      <c r="I64" s="17">
+        <f>ROUND(MAX(G64-IF(G64&gt;=20,7.5,IF(G64&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J64" s="17">
+        <f>ROUND(G64+IF(G64&gt;=20,7.5,IF(G64&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D65" s="21">
+        <f>SUM(D57:D64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="21">
+        <f>SUM(G57:G64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2040  (주식 55% / 채권 45%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D69" s="17" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="E69" s="18">
+        <f>IF(D23&gt;=0.5,(J23-D23)/D23,J23-D23)</f>
+        <v/>
+      </c>
+      <c r="F69" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D69*(1+E69),D69+E69),1.0)</f>
+        <v/>
+      </c>
+      <c r="G69" s="19">
+        <f>ROUND(F69/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H69" s="18">
+        <f>ROUND(G69-D69,2)</f>
+        <v/>
+      </c>
+      <c r="I69" s="17">
+        <f>ROUND(MAX(G69-IF(G69&gt;=20,7.5,IF(G69&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J69" s="17">
+        <f>ROUND(G69+IF(G69&gt;=20,7.5,IF(G69&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D70" s="17" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="E70" s="18">
+        <f>IF(D24&gt;=0.5,(J24-D24)/D24,J24-D24)</f>
+        <v/>
+      </c>
+      <c r="F70" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D70*(1+E70),D70+E70),1.0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="19">
+        <f>ROUND(F70/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H70" s="18">
+        <f>ROUND(G70-D70,2)</f>
+        <v/>
+      </c>
+      <c r="I70" s="17">
+        <f>ROUND(MAX(G70-IF(G70&gt;=20,7.5,IF(G70&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J70" s="17">
+        <f>ROUND(G70+IF(G70&gt;=20,7.5,IF(G70&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D71" s="17" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E71" s="18">
+        <f>IF(D25&gt;=0.5,(J25-D25)/D25,J25-D25)</f>
+        <v/>
+      </c>
+      <c r="F71" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D71*(1+E71),D71+E71),1.0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="19">
+        <f>ROUND(F71/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H71" s="18">
+        <f>ROUND(G71-D71,2)</f>
+        <v/>
+      </c>
+      <c r="I71" s="17">
+        <f>ROUND(MAX(G71-IF(G71&gt;=20,7.5,IF(G71&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J71" s="17">
+        <f>ROUND(G71+IF(G71&gt;=20,7.5,IF(G71&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D72" s="17" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E72" s="18">
+        <f>IF(D26&gt;=0.5,(J26-D26)/D26,J26-D26)</f>
+        <v/>
+      </c>
+      <c r="F72" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D72*(1+E72),D72+E72),1.0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="19">
+        <f>ROUND(F72/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H72" s="18">
+        <f>ROUND(G72-D72,2)</f>
+        <v/>
+      </c>
+      <c r="I72" s="17">
+        <f>ROUND(MAX(G72-IF(G72&gt;=20,7.5,IF(G72&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J72" s="17">
+        <f>ROUND(G72+IF(G72&gt;=20,7.5,IF(G72&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E73" s="18">
+        <f>IF(D27&gt;=0.5,(J27-D27)/D27,J27-D27)</f>
+        <v/>
+      </c>
+      <c r="F73" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D73*(1+E73),D73+E73),1.0)</f>
+        <v/>
+      </c>
+      <c r="G73" s="19">
+        <f>ROUND(F73/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H73" s="18">
+        <f>ROUND(G73-D73,2)</f>
+        <v/>
+      </c>
+      <c r="I73" s="17">
+        <f>ROUND(MAX(G73-IF(G73&gt;=20,7.5,IF(G73&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J73" s="17">
+        <f>ROUND(G73+IF(G73&gt;=20,7.5,IF(G73&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E74" s="18">
+        <f>IF(D28&gt;=0.5,(J28-D28)/D28,J28-D28)</f>
+        <v/>
+      </c>
+      <c r="F74" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D74*(1+E74),D74+E74),1.0)</f>
+        <v/>
+      </c>
+      <c r="G74" s="19">
+        <f>ROUND(F74/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H74" s="18">
+        <f>ROUND(G74-D74,2)</f>
+        <v/>
+      </c>
+      <c r="I74" s="17">
+        <f>ROUND(MAX(G74-IF(G74&gt;=20,7.5,IF(G74&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J74" s="17">
+        <f>ROUND(G74+IF(G74&gt;=20,7.5,IF(G74&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C75" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D75" s="17" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E75" s="18">
+        <f>IF(D29&gt;=0.5,(J29-D29)/D29,J29-D29)</f>
+        <v/>
+      </c>
+      <c r="F75" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D75*(1+E75),D75+E75),1.0)</f>
+        <v/>
+      </c>
+      <c r="G75" s="19">
+        <f>ROUND(F75/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H75" s="18">
+        <f>ROUND(G75-D75,2)</f>
+        <v/>
+      </c>
+      <c r="I75" s="17">
+        <f>ROUND(MAX(G75-IF(G75&gt;=20,7.5,IF(G75&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J75" s="17">
+        <f>ROUND(G75+IF(G75&gt;=20,7.5,IF(G75&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E76" s="18">
+        <f>IF(D30&gt;=0.5,(J30-D30)/D30,J30-D30)</f>
+        <v/>
+      </c>
+      <c r="F76" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D76*(1+E76),D76+E76),1.0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="19">
+        <f>ROUND(F76/SUM(F69:F76)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H76" s="18">
+        <f>ROUND(G76-D76,2)</f>
+        <v/>
+      </c>
+      <c r="I76" s="17">
+        <f>ROUND(MAX(G76-IF(G76&gt;=20,7.5,IF(G76&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J76" s="17">
+        <f>ROUND(G76+IF(G76&gt;=20,7.5,IF(G76&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D77" s="21">
+        <f>SUM(D69:D76)</f>
+        <v/>
+      </c>
+      <c r="G77" s="21">
+        <f>SUM(G69:G76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>TDF 2060  (주식 90% / 채권 10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>지역</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>V.SAA(%)</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Tilt Ratio</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>V.Raw</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>Final(%)</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>vs SAA</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Low(%)</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr">
+        <is>
+          <t>High(%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="n">
+        <v>63</v>
+      </c>
+      <c r="E81" s="18">
+        <f>IF(D23&gt;=0.5,(J23-D23)/D23,J23-D23)</f>
+        <v/>
+      </c>
+      <c r="F81" s="17">
+        <f>MAX(IF(D23&gt;=0.5,D81*(1+E81),D81+E81),1.0)</f>
+        <v/>
+      </c>
+      <c r="G81" s="19">
+        <f>ROUND(F81/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H81" s="18">
+        <f>ROUND(G81-D81,2)</f>
+        <v/>
+      </c>
+      <c r="I81" s="17">
+        <f>ROUND(MAX(G81-IF(G81&gt;=20,7.5,IF(G81&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J81" s="17">
+        <f>ROUND(G81+IF(G81&gt;=20,7.5,IF(G81&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>유럽</t>
+        </is>
+      </c>
+      <c r="D82" s="17" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E82" s="18">
+        <f>IF(D24&gt;=0.5,(J24-D24)/D24,J24-D24)</f>
+        <v/>
+      </c>
+      <c r="F82" s="17">
+        <f>MAX(IF(D24&gt;=0.5,D82*(1+E82),D82+E82),1.0)</f>
+        <v/>
+      </c>
+      <c r="G82" s="19">
+        <f>ROUND(F82/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H82" s="18">
+        <f>ROUND(G82-D82,2)</f>
+        <v/>
+      </c>
+      <c r="I82" s="17">
+        <f>ROUND(MAX(G82-IF(G82&gt;=20,7.5,IF(G82&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J82" s="17">
+        <f>ROUND(G82+IF(G82&gt;=20,7.5,IF(G82&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="D83" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E83" s="18">
+        <f>IF(D25&gt;=0.5,(J25-D25)/D25,J25-D25)</f>
+        <v/>
+      </c>
+      <c r="F83" s="17">
+        <f>MAX(IF(D25&gt;=0.5,D83*(1+E83),D83+E83),1.0)</f>
+        <v/>
+      </c>
+      <c r="G83" s="19">
+        <f>ROUND(F83/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H83" s="18">
+        <f>ROUND(G83-D83,2)</f>
+        <v/>
+      </c>
+      <c r="I83" s="17">
+        <f>ROUND(MAX(G83-IF(G83&gt;=20,7.5,IF(G83&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J83" s="17">
+        <f>ROUND(G83+IF(G83&gt;=20,7.5,IF(G83&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E84" s="18">
+        <f>IF(D26&gt;=0.5,(J26-D26)/D26,J26-D26)</f>
+        <v/>
+      </c>
+      <c r="F84" s="17">
+        <f>MAX(IF(D26&gt;=0.5,D84*(1+E84),D84+E84),1.0)</f>
+        <v/>
+      </c>
+      <c r="G84" s="19">
+        <f>ROUND(F84/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H84" s="18">
+        <f>ROUND(G84-D84,2)</f>
+        <v/>
+      </c>
+      <c r="I84" s="17">
+        <f>ROUND(MAX(G84-IF(G84&gt;=20,7.5,IF(G84&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J84" s="17">
+        <f>ROUND(G84+IF(G84&gt;=20,7.5,IF(G84&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E85" s="18">
+        <f>IF(D27&gt;=0.5,(J27-D27)/D27,J27-D27)</f>
+        <v/>
+      </c>
+      <c r="F85" s="17">
+        <f>MAX(IF(D27&gt;=0.5,D85*(1+E85),D85+E85),1.0)</f>
+        <v/>
+      </c>
+      <c r="G85" s="19">
+        <f>ROUND(F85/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H85" s="18">
+        <f>ROUND(G85-D85,2)</f>
+        <v/>
+      </c>
+      <c r="I85" s="17">
+        <f>ROUND(MAX(G85-IF(G85&gt;=20,7.5,IF(G85&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J85" s="17">
+        <f>ROUND(G85+IF(G85&gt;=20,7.5,IF(G85&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="13" t="inlineStr">
+        <is>
+          <t>주식</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E86" s="18">
+        <f>IF(D28&gt;=0.5,(J28-D28)/D28,J28-D28)</f>
+        <v/>
+      </c>
+      <c r="F86" s="17">
+        <f>MAX(IF(D28&gt;=0.5,D86*(1+E86),D86+E86),1.0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="19">
+        <f>ROUND(F86/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H86" s="18">
+        <f>ROUND(G86-D86,2)</f>
+        <v/>
+      </c>
+      <c r="I86" s="17">
+        <f>ROUND(MAX(G86-IF(G86&gt;=20,7.5,IF(G86&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J86" s="17">
+        <f>ROUND(G86+IF(G86&gt;=20,7.5,IF(G86&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="D87" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E87" s="18">
+        <f>IF(D29&gt;=0.5,(J29-D29)/D29,J29-D29)</f>
+        <v/>
+      </c>
+      <c r="F87" s="17">
+        <f>MAX(IF(D29&gt;=0.5,D87*(1+E87),D87+E87),1.0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="19">
+        <f>ROUND(F87/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H87" s="18">
+        <f>ROUND(G87-D87,2)</f>
+        <v/>
+      </c>
+      <c r="I87" s="17">
+        <f>ROUND(MAX(G87-IF(G87&gt;=20,7.5,IF(G87&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J87" s="17">
+        <f>ROUND(G87+IF(G87&gt;=20,7.5,IF(G87&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="13" t="inlineStr">
+        <is>
+          <t>채권</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E88" s="18">
+        <f>IF(D30&gt;=0.5,(J30-D30)/D30,J30-D30)</f>
+        <v/>
+      </c>
+      <c r="F88" s="17">
+        <f>MAX(IF(D30&gt;=0.5,D88*(1+E88),D88+E88),1.0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="19">
+        <f>ROUND(F88/SUM(F81:F88)*100,2)</f>
+        <v/>
+      </c>
+      <c r="H88" s="18">
+        <f>ROUND(G88-D88,2)</f>
+        <v/>
+      </c>
+      <c r="I88" s="17">
+        <f>ROUND(MAX(G88-IF(G88&gt;=20,7.5,IF(G88&gt;=10,5.0,2.5)),0),2)</f>
+        <v/>
+      </c>
+      <c r="J88" s="17">
+        <f>ROUND(G88+IF(G88&gt;=20,7.5,IF(G88&gt;=10,5.0,2.5)),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="20" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="D89" s="21">
+        <f>SUM(D81:D88)</f>
+        <v/>
+      </c>
+      <c r="G89" s="21">
+        <f>SUM(G81:G88)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add dampened tilt power parameter
</commit_message>
<xml_diff>
--- a/TAA_Dashboard.xlsx
+++ b/TAA_Dashboard.xlsx
@@ -686,6 +686,19 @@
       </c>
     </row>
     <row r="7">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Tilt Power (p)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>← 0=균등, 0.5=감쇠, 1=비례</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Neutral</t>
@@ -1132,7 +1145,7 @@
         <v/>
       </c>
       <c r="H26" s="22">
-        <f>G26*$C$6</f>
+        <f>(G26/(SUMIF($B$26:$B$33,B26,$G$26:$G$33)/COUNTIF($B$26:$B$33,B26)))^$C$7*(SUMIF($B$26:$B$33,B26,$G$26:$G$33)/COUNTIF($B$26:$B$33,B26))*$C$6</f>
         <v/>
       </c>
       <c r="I26" s="23">
@@ -1182,7 +1195,7 @@
         <v/>
       </c>
       <c r="H27" s="22">
-        <f>G27*$C$6</f>
+        <f>(G27/(SUMIF($B$26:$B$33,B27,$G$26:$G$33)/COUNTIF($B$26:$B$33,B27)))^$C$7*(SUMIF($B$26:$B$33,B27,$G$26:$G$33)/COUNTIF($B$26:$B$33,B27))*$C$6</f>
         <v/>
       </c>
       <c r="I27" s="23">
@@ -1232,7 +1245,7 @@
         <v/>
       </c>
       <c r="H28" s="22">
-        <f>G28*$C$6</f>
+        <f>(G28/(SUMIF($B$26:$B$33,B28,$G$26:$G$33)/COUNTIF($B$26:$B$33,B28)))^$C$7*(SUMIF($B$26:$B$33,B28,$G$26:$G$33)/COUNTIF($B$26:$B$33,B28))*$C$6</f>
         <v/>
       </c>
       <c r="I28" s="23">
@@ -1282,7 +1295,7 @@
         <v/>
       </c>
       <c r="H29" s="22">
-        <f>G29*$C$6</f>
+        <f>(G29/(SUMIF($B$26:$B$33,B29,$G$26:$G$33)/COUNTIF($B$26:$B$33,B29)))^$C$7*(SUMIF($B$26:$B$33,B29,$G$26:$G$33)/COUNTIF($B$26:$B$33,B29))*$C$6</f>
         <v/>
       </c>
       <c r="I29" s="23">
@@ -1332,7 +1345,7 @@
         <v/>
       </c>
       <c r="H30" s="22">
-        <f>G30*$C$6</f>
+        <f>(G30/(SUMIF($B$26:$B$33,B30,$G$26:$G$33)/COUNTIF($B$26:$B$33,B30)))^$C$7*(SUMIF($B$26:$B$33,B30,$G$26:$G$33)/COUNTIF($B$26:$B$33,B30))*$C$6</f>
         <v/>
       </c>
       <c r="I30" s="23">
@@ -1382,7 +1395,7 @@
         <v/>
       </c>
       <c r="H31" s="22">
-        <f>G31*$C$6</f>
+        <f>(G31/(SUMIF($B$26:$B$33,B31,$G$26:$G$33)/COUNTIF($B$26:$B$33,B31)))^$C$7*(SUMIF($B$26:$B$33,B31,$G$26:$G$33)/COUNTIF($B$26:$B$33,B31))*$C$6</f>
         <v/>
       </c>
       <c r="I31" s="23">
@@ -1432,7 +1445,7 @@
         <v/>
       </c>
       <c r="H32" s="22">
-        <f>G32*$C$6</f>
+        <f>(G32/(SUMIF($B$26:$B$33,B32,$G$26:$G$33)/COUNTIF($B$26:$B$33,B32)))^$C$7*(SUMIF($B$26:$B$33,B32,$G$26:$G$33)/COUNTIF($B$26:$B$33,B32))*$C$6</f>
         <v/>
       </c>
       <c r="I32" s="23">
@@ -1482,7 +1495,7 @@
         <v/>
       </c>
       <c r="H33" s="22">
-        <f>G33*$C$6</f>
+        <f>(G33/(SUMIF($B$26:$B$33,B33,$G$26:$G$33)/COUNTIF($B$26:$B$33,B33)))^$C$7*(SUMIF($B$26:$B$33,B33,$G$26:$G$33)/COUNTIF($B$26:$B$33,B33))*$C$6</f>
         <v/>
       </c>
       <c r="I33" s="23">
@@ -1916,7 +1929,7 @@
     <row r="57">
       <c r="B57" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Tilt_i = Base_i × Tilt Rate</t>
+          <t xml:space="preserve">  3. Tilt_i = (Base_i / avg_Base)^p × avg_Base × Tilt Rate</t>
         </is>
       </c>
     </row>

</xml_diff>